<commit_message>
Update documentation to reflect recent data rescue and merge checklist changes
Update the title of the Final Gap Analysis document and the description of the Duplicate Merge Checklist to reflect the updated number of duplicate pairs.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ef7bf022-0b3a-4156-9c38-2b98b837c1d1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 5fd5733a-2940-431e-824f-199493293829
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e9fe007f-c11f-42ca-a1dd-347ccc032e17/ef7bf022-0b3a-4156-9c38-2b98b837c1d1/p7QEcg3
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/docs/CAS_Duplicate_Merge_Checklist_2026-05-07.xlsx
+++ b/docs/CAS_Duplicate_Merge_Checklist_2026-05-07.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -407,7 +407,7 @@
     <col min="5" max="5" width="60.83203125" customWidth="1"/>
     <col min="6" max="6" width="24.83203125" customWidth="1"/>
     <col min="7" max="7" width="60.83203125" customWidth="1"/>
-    <col min="8" max="8" width="55.83203125" customWidth="1"/>
+    <col min="8" max="8" width="60.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -434,7 +434,7 @@
         <v>DELETE — Click to open</v>
       </c>
       <c r="H1" t="str">
-        <v>Action</v>
+        <v>Note</v>
       </c>
       <c r="I1" t="str">
         <v>Status (Jan to fill)</v>
@@ -463,7 +463,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002296017</v>
       </c>
       <c r="H2" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -492,7 +492,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002297006</v>
       </c>
       <c r="H3" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -521,7 +521,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002298013</v>
       </c>
       <c r="H4" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -550,7 +550,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002303017</v>
       </c>
       <c r="H5" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -579,7 +579,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002297008</v>
       </c>
       <c r="H6" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -608,7 +608,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002307023</v>
       </c>
       <c r="H7" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -637,7 +637,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002305021</v>
       </c>
       <c r="H8" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -666,7 +666,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002305023</v>
       </c>
       <c r="H9" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -695,7 +695,7 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002298015</v>
       </c>
       <c r="H10" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I10" t="str">
         <v/>
@@ -724,22 +724,80 @@
         <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002307021</v>
       </c>
       <c r="H11" t="str">
-        <v>Open BOTH, verify identical, then DELETE the right-hand one</v>
+        <v>Original was synced via background worker; dup from re-submit</v>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Emilie Theberge</v>
+      </c>
+      <c r="C12" t="str">
+        <v>emilie.theberge@ubc.ca</v>
+      </c>
+      <c r="D12" t="str">
+        <v>6999043000002288015</v>
+      </c>
+      <c r="E12" t="str">
+        <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002288015</v>
+      </c>
+      <c r="F12" t="str">
+        <v>6999043000002305026</v>
+      </c>
+      <c r="G12" t="str">
+        <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002305026</v>
+      </c>
+      <c r="H12" t="str">
+        <v>BOTH from May 8 rescue (script ran twice)</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Niloufar Ahmadbeigi</v>
+      </c>
+      <c r="C13" t="str">
+        <v>ahmadbeigi@hhsc.ca</v>
+      </c>
+      <c r="D13" t="str">
+        <v>6999043000002288014</v>
+      </c>
+      <c r="E13" t="str">
+        <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002288014</v>
+      </c>
+      <c r="F13" t="str">
+        <v>6999043000002291032</v>
+      </c>
+      <c r="G13" t="str">
+        <v>https://crm.zoho.com/crm/org/tab/Leads/6999043000002291032</v>
+      </c>
+      <c r="H13" t="str">
+        <v>BOTH from May 8 rescue (script ran twice)</v>
+      </c>
+      <c r="I13" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="120.83203125" customWidth="1"/>
@@ -774,7 +832,7 @@
         <v>2a</v>
       </c>
       <c r="B4" t="str">
-        <v>Click the "KEEP — Click to open" link. Verify the record looks correct (this is the OLDER one, created via background worker).</v>
+        <v>Click the "KEEP — Click to open" link to verify the older record.</v>
       </c>
     </row>
     <row r="5">
@@ -782,7 +840,7 @@
         <v>2b</v>
       </c>
       <c r="B5" t="str">
-        <v>Click the "DELETE — Click to open" link. Verify it has identical name + email (it is the duplicate from re-submit).</v>
+        <v>Click the "DELETE — Click to open" link to verify it has the same name + email.</v>
       </c>
     </row>
     <row r="6">
@@ -790,7 +848,7 @@
         <v>2c</v>
       </c>
       <c r="B6" t="str">
-        <v>Optional: in Zoho, use Settings → Data Administration → Find Duplicates by Email if you prefer the bulk merge UI.</v>
+        <v>Optional: Use Zoho Settings → Data Administration → Find Duplicates by Email for bulk handling.</v>
       </c>
     </row>
     <row r="7">
@@ -798,7 +856,7 @@
         <v>2d</v>
       </c>
       <c r="B7" t="str">
-        <v>Delete the duplicate record (or use Zoho Merge to combine, keeping the older).</v>
+        <v>Delete the duplicate (or use Zoho Merge to combine, keeping the older).</v>
       </c>
     </row>
     <row r="8">
@@ -806,7 +864,7 @@
         <v>2e</v>
       </c>
       <c r="B8" t="str">
-        <v>Mark the row Status as "DONE" so you can track progress.</v>
+        <v>Mark Status as "DONE" so you can track progress.</v>
       </c>
     </row>
     <row r="9">
@@ -814,7 +872,7 @@
         <v>3</v>
       </c>
       <c r="B9" t="str">
-        <v>After all 10 pairs are merged, total Lead count should drop from 298 → 288.</v>
+        <v>After all 12 pairs are merged, total Lead count should drop from 303 → 291.</v>
       </c>
     </row>
     <row r="10">
@@ -822,12 +880,20 @@
         <v>4</v>
       </c>
       <c r="B10" t="str">
-        <v>Note: Mary O'Sullivan also has a 3rd record (#264 sub) that was already manually pushed in a prior session — check for that too.</v>
+        <v>Note: Mary O'Sullivan also has a 3rd record (#264 sub) manually pushed in a prior session — also check for that.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>5</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Note: Emilie + Niloufar were both pushed twice during the May 8 rescue (the script was rerun before the first result was visible). Both copies are in CRM and need merging.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>